<commit_message>
Restore separated S3 rate presentation
</commit_message>
<xml_diff>
--- a/assets/MUD_Water_Analysis.xlsx
+++ b/assets/MUD_Water_Analysis.xlsx
@@ -29,7 +29,7 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="409" uniqueCount="358">
   <si>
-    <t xml:space="preserve">Grand Lakes MUD 2 - Account 30402-0600812002 - 3923 Rose Grove Ln, Katy TX</t>
+    <t xml:space="preserve">Grand Lakes MUD 2 - Account 30402-0600812002 - author home Rose Grove Ln, Katy TX</t>
   </si>
   <si>
     <t xml:space="preserve">Every bill transcribed from the scanned images. Blue = read off the bill. Black = calculated by formula.</t>
@@ -551,7 +551,7 @@
     <t xml:space="preserve">S2 vs Current</t>
   </si>
   <si>
-    <t xml:space="preserve">Neighbor at 3918 / your own low months</t>
+    <t xml:space="preserve">Neighbor at nearby home / your own low months</t>
   </si>
   <si>
     <t xml:space="preserve">Your 2021-2025 typical month</t>
@@ -608,7 +608,7 @@
     <t xml:space="preserve">&gt;50k</t>
   </si>
   <si>
-    <t xml:space="preserve">27% of homes use &lt;10k/month (bills ~$60-79 all-in today) - the $80 neighbor at 3918 is one of 180 such homes, using ~7k gal. Your July 2026 (24k) is in roughly the top 15% of meters. Your pre-2026 median (~9-10k) was typical.</t>
+    <t xml:space="preserve">27% of homes use &lt;10k/month (bills ~$60-79 all-in today) - the $80 neighbor at nearby home is one of 180 such homes, using ~7k gal. Your July 2026 (24k) is in roughly the top 15% of meters. Your pre-2026 median (~9-10k) was typical.</t>
   </si>
   <si>
     <t xml:space="preserve">FY27 proposed budget W+WW revenue = $950,922 = EXACTLY Scenario 1 projected service revenue -&gt; board leaning Scenario 1 now, second-phase increase 2028, $100 fee held in reserve. FY27 budget also carries $150,000 for PUC Appeal - district expects a challenge.</t>
@@ -716,7 +716,7 @@
     <t xml:space="preserve">true low user (38 homes)</t>
   </si>
   <si>
-    <t xml:space="preserve">neighbor at 3918 / your low months</t>
+    <t xml:space="preserve">neighbor at nearby home / your low months</t>
   </si>
   <si>
     <t xml:space="preserve">your normal month</t>
@@ -851,7 +851,7 @@
     <t xml:space="preserve">COS vs S1</t>
   </si>
   <si>
-    <t xml:space="preserve">neighbor at 3918</t>
+    <t xml:space="preserve">neighbor at nearby home</t>
   </si>
   <si>
     <t xml:space="preserve">your July 2026</t>

</xml_diff>